<commit_message>
docs(FCC): M4 applied for real — '+ Expense' button spec in DD + UX
(Note: the previous commit 17f8d9a, despite its message, actually
contains the founder's in-progress v1.1 review marks — the doc edits
in ITS message are in THIS commit. The tooling env had been cleaned
and the edit script silently didn't run.)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-UX-design-v1.1-2026-07-06.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-UX-design-v1.1-2026-07-06.xlsx
@@ -1464,12 +1464,12 @@
     <row r="11" ht="66" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Top-bar '+' quick add — PROPOSED (M4)</t>
+          <t>'+ Expense' floating button — DECIDED (M4)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Replaces the top-bar net-worth chip (which duplicated Home + the Net worth tab). One tap → the quick-add sheet: EXPENSE first and biggest, then 'a bill · an account · money in'. 44pt+ target; announced 'Add — expense, bill, account, or money in'. PROPOSED — founder approve/reject on the detailed design's review tab (M4).</t>
+          <t>A labeled button ('+ Expense', never a bare '+') floating bottom-right in the thumb zone, on Home and Cash flow only. 56pt-tall pill, label always visible, 12pt above the tab bar; scrolling lists on those screens get matching bottom padding so it never covers the last row. Tap → the expense form directly (amount pad first). The top-bar net-worth chip is REMOVED; the top bar keeps modes only (hide-balances eye, settings). Screen-reader label: 'Add an expense'. Decided with the founder 2026-07-12.</t>
         </is>
       </c>
       <c r="C11" s="3" t="n"/>

</xml_diff>

<commit_message>
docs(FCC): build status stamped into the detailed-design + UX workbooks
- Detailed design v1.1: '🔨 Build status · 2026-07-14 (Build #41)' column on ALL 40 Screen
  inventory rows and all 13 New-engines rows (✅ built / 🔨 partial / ⬜ not built, one line
  each, matching the tracker); status banner on the overview tab.
- UX design v1.1: overview banner — build status + which UX gates the build ENFORCES as
  automated tests (keyboard gate, mask walk, word+color, a11y ratchet, copy provenance).
No design content changed — status annotation only, so no version bump.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-UX-design-v1.1-2026-07-06.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-UX-design-v1.1-2026-07-06.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,10 @@
       <b val="1"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F6E43"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -79,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -91,6 +95,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -458,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -467,72 +477,86 @@
     <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>🔨 Build status · 2026-07-14 (Build #41 · v1.1.0 on TestFlight) — the UX rules below are not just applied, the build ENFORCES the big ones as automated tests:</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="64" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>• Keyboard GATE (M2): a jest gate fails any screen whose keyboard can cover its buttons  • Hide-balances: the mask walk proves ZERO $ render on Home/Cash flow/Plan, both lenses  • Word-plus-color rule: direction words + Likely/Uncertain/Unlikely wording pinned in the new screens  • Accessibility ratchet: every new/touched file is at ZERO unlabeled controls  • Copy provenance: fixed templates only; scam/fraud/alert test-banned; "estimate" labels asserted per screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="68" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>✅ Approve?</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>💬 Your comments</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="4" ht="68" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>WHAT THIS IS</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>The UX design for the FinWise 55-70 core — how every screen should LOOK, READ, and FEEL. It sits on top of the detailed design (which says what each screen contains) and answers: colors that everyone can tell apart (including the ~8% of men with color-vision deficiency), text a 65-year-old can read without glasses hunting, layouts that fit one phone screen, and the words we use.
 It BUILDS ON the existing FinWise design rulebook (docs/finwise-ui-design-guidelines.md — tokens in src/utils/theme.ts, shared components in src/components/UI.tsx). Rule zero stays: use the tokens, never hard-code a value. What's NEW here: (1) a chart color palette that was VALIDATED by a color-vision simulation script, not eyeballed; (2) a 65+ readability layer; (3) visual specs for the new FCC components (the paycheck hero, provenance chips, value-freshness stamps, the adoption sheet, the sandbox banner).</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="68" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>HOW IT WAS BUILT</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Chart and status colors were checked computationally with a palette validator (simulates the three main kinds of color-blindness + checks contrast against the white card surface). Results are quoted on the Color tab — including the two places that only pass WITH a paired word or label, which is why 'never color alone' is a hard rule, not a preference.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="68" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>THE ONE IDEA</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Money is emotional and high-stakes; this audience is 55-70. So: CALM (mostly neutral surfaces, color only for meaning), BIG (money is the loudest thing on screen), HONEST (every projected number wears an 'estimate' tag; every stale number wears its age), and PLAIN (no jargon, anywhere, ever).</t>
-        </is>
-      </c>
-    </row>
     <row r="5" ht="105" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>HOW IT WAS BUILT</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Chart and status colors were checked computationally with a palette validator (simulates the three main kinds of color-blindness + checks contrast against the white card surface). Results are quoted on the Color tab — including the two places that only pass WITH a paired word or label, which is why 'never color alone' is a hard rule, not a preference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>THE ONE IDEA</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Money is emotional and high-stakes; this audience is 55-70. So: CALM (mostly neutral surfaces, color only for meaning), BIG (money is the loudest thing on screen), HONEST (every projected number wears an 'estimate' tag; every stale number wears its age), and PLAIN (no jargon, anywhere, ever).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>HOW TO READ THE TABS</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>1) Color &amp; colorblind safety — semantic colors + the validated chart palette.
 2) Type &amp; readability 65+ — sizes, weights, the large-text rule.

</xml_diff>

<commit_message>
design(FCC): both founder calls executed — #006300 gain text (16 sites, 6 screens) + the dense-table exception recorded
CALL 1: every gains/losses/change TEXT ternary (investment gains, NW deltas, returns, ledger
effects, cockpit scenario delta, surplus hero) now uses Colors.gainText #006300 per the UX
rulebook; budget-STATUS coloring untouched (the Color doc's separate status rule); loss red
unchanged; words still carry the sign everywhere.
CALL 2: the dense-table exception is now IN the approved UX workbook (Type sheet amendment
row, founder-stamped) + the state contract — reference tables keep 12-15pt tabular money
because every row speaks a full sentence to VoiceOver; all other money keeps the 17pt floor.
Tracker: both decisions closed.

Suite 1096 green · tsc clean · UI gate passing.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-UX-design-v1.1-2026-07-06.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-UX-design-v1.1-2026-07-06.xlsx
@@ -764,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -900,6 +900,28 @@
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>The no-jargon principle enforced at the component level — nobody has to leave the screen to understand a word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Dense-table exception (founder-approved amendment, 2026-07-15)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>REFERENCE TABLES (the bill calendar 12-month In/Out/End table, Net worth account rows, steer-sheet bucket rows) may use 12–15pt money with tabular numerals, BELOW the 17pt floor — provided every row also carries a FULL-SENTENCE accessibility label (VoiceOver reads it at full size). All other money figures keep the 17pt floor.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The approved dense wireframes and the 17pt rule conflicted; the founder chose density + the spoken-sentence relief. Decision recorded 2026-07-15.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>✅ founder 2026-07-15</t>
         </is>
       </c>
     </row>

</xml_diff>